<commit_message>
fix(inventario): paneles JA 620 corregidos a 1546 (eran 15)
Cliente confirma que el numero real de paneles JA Solar Bifacial 620W
en stock es 1546, no 15 como aparece en el Excel original (error de
captura).

- Agregada estructura CORRECCIONES_LOTES en limpiar_inventario.py para
  documentar correcciones del cliente sin tocar el archivo original
  (auditoria preservada en hoja 'Lotes detalle' que ahora muestra
  cantidad original vs corregida con motivo en columna nueva).
- Hoja 'Estructura PV' resalta el stock corregido en amarillo y agrega
  comment con la justificacion.

Impacto en valuacion:
  Estructura PV   : $94,320 -> $212,023 USD (+$117,703)
  GRAN TOTAL inv. : $118,808 -> $236,512 USD = $4,080,537 MXN @ TC actual

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/inventario/inventario-consolidado.xlsx
+++ b/data/inventario/inventario-consolidado.xlsx
@@ -73,7 +73,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +88,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001A1A2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -122,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -137,11 +142,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -216,6 +223,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Sistema</author>
+  </authors>
+  <commentList>
+    <comment ref="C2" authorId="0" shapeId="0">
+      <text>
+        <t>Stock corregido por instrucción del cliente. Ver hoja 'Lotes detalle'.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -786,22 +808,22 @@
         </is>
       </c>
       <c r="C2" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="D2" s="10" t="n">
+        <v>1546</v>
+      </c>
+      <c r="D2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="E2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F2" s="11" t="n">
+      <c r="F2" s="12" t="n">
         <v>76.88</v>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="13">
         <f>C2*F2</f>
         <v/>
       </c>
-      <c r="H2" s="12">
+      <c r="H2" s="13">
         <f>G2*tc_actual</f>
         <v/>
       </c>
@@ -817,23 +839,23 @@
           <t>Ángulo-Riel 4.0m, Alu 6105-T6</t>
         </is>
       </c>
-      <c r="C3" s="10" t="n">
+      <c r="C3" s="11" t="n">
         <v>450</v>
       </c>
-      <c r="D3" s="10" t="n">
+      <c r="D3" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="11" t="n">
+      <c r="F3" s="12" t="n">
         <v>25.25</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="13">
         <f>C3*F3</f>
         <v/>
       </c>
-      <c r="H3" s="12">
+      <c r="H3" s="13">
         <f>G3*tc_actual</f>
         <v/>
       </c>
@@ -849,23 +871,23 @@
           <t>2 Abrazaderas universales de Aluminio para paneles de 30-46mm</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="11" t="n">
         <v>3045</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="11" t="n">
+      <c r="F4" s="12" t="n">
         <v>3.9879</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="13">
         <f>C4*F4</f>
         <v/>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="13">
         <f>G4*tc_actual</f>
         <v/>
       </c>
@@ -881,23 +903,23 @@
           <t>4 Clips de conexión para Next Rail</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="11" t="n">
         <v>1440</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="12" t="n">
         <v>6.05</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="13">
         <f>C5*F5</f>
         <v/>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="13">
         <f>G5*tc_actual</f>
         <v/>
       </c>
@@ -913,23 +935,23 @@
           <t>Terminal de conexión a tierra para 2 cables, Next Rail con certificiación UL.</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="11" t="n">
         <v>950</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="12" t="n">
         <v>2.19</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="13">
         <f>C6*F6</f>
         <v/>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="13">
         <f>G6*tc_actual</f>
         <v/>
       </c>
@@ -945,23 +967,23 @@
           <t>1 Soporte "L" de 95 mm de altura para Nxt-Rail</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="11" t="n">
         <v>645</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="12" t="n">
         <v>2.1751</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="13">
         <f>C7*F7</f>
         <v/>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="13">
         <f>G7*tc_actual</f>
         <v/>
       </c>
@@ -977,23 +999,23 @@
           <t>1 empalme de riel con puesta a tierra para Next Rail NXT-RX.</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="11" t="n">
         <v>1215</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="12" t="n">
         <v>2.7874</v>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="13">
         <f>C8*F8</f>
         <v/>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="13">
         <f>G8*tc_actual</f>
         <v/>
       </c>
@@ -1009,23 +1031,23 @@
           <t>Perfil NetRail 4.80m, mill finish, Aluminio 6105-T6</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <v>1120</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F9" s="12" t="n">
         <v>25.5953</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="13">
         <f>C9*F9</f>
         <v/>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="13">
         <f>G9*tc_actual</f>
         <v/>
       </c>
@@ -1041,23 +1063,23 @@
           <t>5 Tbolt M8x25 Acero Inoxidable con tuerca para NextRail</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="11" t="n">
         <v>1500</v>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="12" t="n">
         <v>2.47</v>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="13">
         <f>C10*F10</f>
         <v/>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="13">
         <f>G10*tc_actual</f>
         <v/>
       </c>
@@ -1073,23 +1095,23 @@
           <t>1 Conector para riel inclinado</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="11" t="n">
         <v>1215</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="12" t="n">
         <v>3.1748</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="13">
         <f>C11*F11</f>
         <v/>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="13">
         <f>G11*tc_actual</f>
         <v/>
       </c>
@@ -1105,23 +1127,23 @@
           <t>10 Conectores MC4, 5 Hembras y 5 Macho cable 14-10AWG, 1500 Vdc</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="12" t="n">
         <v>5.56</v>
       </c>
-      <c r="G12" s="12">
+      <c r="G12" s="13">
         <f>C12*F12</f>
         <v/>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="13">
         <f>G12*tc_actual</f>
         <v/>
       </c>
@@ -1137,23 +1159,23 @@
           <t>Cable Fotovoltaico negro PV Wire carrete 762 mts 10AWG 2000V De 19 hilos</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F13" s="12" t="n">
         <v>612.8200000000001</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="13">
         <f>C13*F13</f>
         <v/>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="13">
         <f>G13*tc_actual</f>
         <v/>
       </c>
@@ -1169,49 +1191,50 @@
           <t>Cable Fotovoltaico Negro PV wire carrete 762 mts 12AWG 2000V de 19 hilos</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="11" t="n">
+      <c r="F14" s="12" t="n">
         <v>421.81</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="13">
         <f>C14*F14</f>
         <v/>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="13">
         <f>G14*tc_actual</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="n"/>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="A15" s="14" t="n"/>
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n"/>
-      <c r="D15" s="13" t="n"/>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="13" t="n"/>
-      <c r="G15" s="14">
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="14" t="n"/>
+      <c r="E15" s="14" t="n"/>
+      <c r="F15" s="14" t="n"/>
+      <c r="G15" s="15">
         <f>SUM(G2:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="14">
+      <c r="H15" s="15">
         <f>SUM(H2:H14)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1332,28 +1355,28 @@
           <t>CAL 10</t>
         </is>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="F2" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="10" t="n">
+      <c r="G2" s="11" t="n">
         <v>256</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="11" t="n">
         <v>206</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="11">
         <f>F2+G2-H2</f>
         <v/>
       </c>
-      <c r="J2" s="11" t="n"/>
-      <c r="K2" s="12" t="n">
+      <c r="J2" s="12" t="n"/>
+      <c r="K2" s="13" t="n">
         <v>26.28</v>
       </c>
-      <c r="L2" s="12">
+      <c r="L2" s="13">
         <f>I2*K2</f>
         <v/>
       </c>
-      <c r="M2" s="12">
+      <c r="M2" s="13">
         <f>L2*tc_actual</f>
         <v/>
       </c>
@@ -1384,28 +1407,28 @@
           <t>2 kW</t>
         </is>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="F3" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="10" t="n">
+      <c r="G3" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="11">
         <f>F3+G3-H3</f>
         <v/>
       </c>
-      <c r="J3" s="11" t="n"/>
-      <c r="K3" s="12" t="n">
+      <c r="J3" s="12" t="n"/>
+      <c r="K3" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L3" s="12">
+      <c r="L3" s="13">
         <f>I3*K3</f>
         <v/>
       </c>
-      <c r="M3" s="12">
+      <c r="M3" s="13">
         <f>L3*tc_actual</f>
         <v/>
       </c>
@@ -1436,28 +1459,28 @@
           <t>PARA 100</t>
         </is>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="F4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="G4" s="11" t="n">
         <v>73</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="11" t="n">
         <v>54</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="11">
         <f>F4+G4-H4</f>
         <v/>
       </c>
-      <c r="J4" s="11" t="n"/>
-      <c r="K4" s="12" t="n">
+      <c r="J4" s="12" t="n"/>
+      <c r="K4" s="13" t="n">
         <v>141.16</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="13">
         <f>I4*K4</f>
         <v/>
       </c>
-      <c r="M4" s="12">
+      <c r="M4" s="13">
         <f>L4*tc_actual</f>
         <v/>
       </c>
@@ -1488,28 +1511,28 @@
           <t>CAL 10</t>
         </is>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="F5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="11" t="n">
         <v>82</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="11">
         <f>F5+G5-H5</f>
         <v/>
       </c>
-      <c r="J5" s="11" t="n"/>
-      <c r="K5" s="12" t="n">
+      <c r="J5" s="12" t="n"/>
+      <c r="K5" s="13" t="n">
         <v>5.77</v>
       </c>
-      <c r="L5" s="12">
+      <c r="L5" s="13">
         <f>I5*K5</f>
         <v/>
       </c>
-      <c r="M5" s="12">
+      <c r="M5" s="13">
         <f>L5*tc_actual</f>
         <v/>
       </c>
@@ -1540,30 +1563,30 @@
           <t>2 kW</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="G6" s="11" t="n">
         <v>186</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="11" t="n">
         <v>184</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="11">
         <f>F6+G6-H6</f>
         <v/>
       </c>
-      <c r="J6" s="11" t="n">
+      <c r="J6" s="12" t="n">
         <v>0.1286</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="K6" s="13" t="n">
         <v>257.24</v>
       </c>
-      <c r="L6" s="12">
+      <c r="L6" s="13">
         <f>I6*K6</f>
         <v/>
       </c>
-      <c r="M6" s="12">
+      <c r="M6" s="13">
         <f>L6*tc_actual</f>
         <v/>
       </c>
@@ -1594,30 +1617,30 @@
           <t>1.05 kW</t>
         </is>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="11" t="n">
         <v>76</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I7" s="11">
         <f>F7+G7-H7</f>
         <v/>
       </c>
-      <c r="J7" s="11" t="n">
+      <c r="J7" s="12" t="n">
         <v>0.1835</v>
       </c>
-      <c r="K7" s="12" t="n">
+      <c r="K7" s="13" t="n">
         <v>192.67</v>
       </c>
-      <c r="L7" s="12">
+      <c r="L7" s="13">
         <f>I7*K7</f>
         <v/>
       </c>
-      <c r="M7" s="12">
+      <c r="M7" s="13">
         <f>L7*tc_actual</f>
         <v/>
       </c>
@@ -1648,30 +1671,30 @@
           <t>3 kW</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="H8" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I8" s="11">
         <f>F8+G8-H8</f>
         <v/>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="J8" s="12" t="n">
         <v>0.125</v>
       </c>
-      <c r="K8" s="12" t="n">
+      <c r="K8" s="13" t="n">
         <v>375</v>
       </c>
-      <c r="L8" s="12">
+      <c r="L8" s="13">
         <f>I8*K8</f>
         <v/>
       </c>
-      <c r="M8" s="12">
+      <c r="M8" s="13">
         <f>L8*tc_actual</f>
         <v/>
       </c>
@@ -1702,30 +1725,30 @@
           <t>5 kW</t>
         </is>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F9" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="10" t="n">
+      <c r="H9" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="11">
         <f>F9+G9-H9</f>
         <v/>
       </c>
-      <c r="J9" s="11" t="n">
+      <c r="J9" s="12" t="n">
         <v>0.1033</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="K9" s="13" t="n">
         <v>516.4</v>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="13">
         <f>I9*K9</f>
         <v/>
       </c>
-      <c r="M9" s="12">
+      <c r="M9" s="13">
         <f>L9*tc_actual</f>
         <v/>
       </c>
@@ -1756,30 +1779,30 @@
           <t>7 kW</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="F10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G10" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="H10" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="11">
         <f>F10+G10-H10</f>
         <v/>
       </c>
-      <c r="J10" s="11" t="n">
+      <c r="J10" s="12" t="n">
         <v>0.1093</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="K10" s="13" t="n">
         <v>765.35</v>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="13">
         <f>I10*K10</f>
         <v/>
       </c>
-      <c r="M10" s="12">
+      <c r="M10" s="13">
         <f>L10*tc_actual</f>
         <v/>
       </c>
@@ -1810,30 +1833,30 @@
           <t>9 kW</t>
         </is>
       </c>
-      <c r="F11" s="10" t="n">
+      <c r="F11" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="10" t="n">
+      <c r="G11" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="11">
         <f>F11+G11-H11</f>
         <v/>
       </c>
-      <c r="J11" s="11" t="n">
+      <c r="J11" s="12" t="n">
         <v>0.093</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="K11" s="13" t="n">
         <v>836.73</v>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="13">
         <f>I11*K11</f>
         <v/>
       </c>
-      <c r="M11" s="12">
+      <c r="M11" s="13">
         <f>L11*tc_actual</f>
         <v/>
       </c>
@@ -1864,30 +1887,30 @@
           <t>8.5 kW</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n">
+      <c r="F12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="10" t="n">
+      <c r="G12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="10" t="n">
+      <c r="H12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="11">
         <f>F12+G12-H12</f>
         <v/>
       </c>
-      <c r="J12" s="11" t="n">
+      <c r="J12" s="12" t="n">
         <v>0.1024</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="K12" s="13" t="n">
         <v>870</v>
       </c>
-      <c r="L12" s="12">
+      <c r="L12" s="13">
         <f>I12*K12</f>
         <v/>
       </c>
-      <c r="M12" s="12">
+      <c r="M12" s="13">
         <f>L12*tc_actual</f>
         <v/>
       </c>
@@ -1918,30 +1941,30 @@
           <t>11.4 kW</t>
         </is>
       </c>
-      <c r="F13" s="10" t="n">
+      <c r="F13" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="10" t="n">
+      <c r="G13" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="10" t="n">
+      <c r="H13" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="11">
         <f>F13+G13-H13</f>
         <v/>
       </c>
-      <c r="J13" s="11" t="n">
+      <c r="J13" s="12" t="n">
         <v>0.0876</v>
       </c>
-      <c r="K13" s="12" t="n">
+      <c r="K13" s="13" t="n">
         <v>999</v>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="13">
         <f>I13*K13</f>
         <v/>
       </c>
-      <c r="M13" s="12">
+      <c r="M13" s="13">
         <f>L13*tc_actual</f>
         <v/>
       </c>
@@ -1972,30 +1995,30 @@
           <t>5 kW</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="F14" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="10" t="n">
+      <c r="G14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="10" t="n">
+      <c r="H14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="I14" s="10">
+      <c r="I14" s="11">
         <f>F14+G14-H14</f>
         <v/>
       </c>
-      <c r="J14" s="11" t="n">
+      <c r="J14" s="12" t="n">
         <v>0.135</v>
       </c>
-      <c r="K14" s="12" t="n">
+      <c r="K14" s="13" t="n">
         <v>675</v>
       </c>
-      <c r="L14" s="12">
+      <c r="L14" s="13">
         <f>I14*K14</f>
         <v/>
       </c>
-      <c r="M14" s="12">
+      <c r="M14" s="13">
         <f>L14*tc_actual</f>
         <v/>
       </c>
@@ -2026,30 +2049,30 @@
           <t>6 kW</t>
         </is>
       </c>
-      <c r="F15" s="10" t="n">
+      <c r="F15" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="10" t="n">
+      <c r="G15" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="H15" s="10" t="n">
+      <c r="H15" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="I15" s="10">
+      <c r="I15" s="11">
         <f>F15+G15-H15</f>
         <v/>
       </c>
-      <c r="J15" s="11" t="n">
+      <c r="J15" s="12" t="n">
         <v>0.1175</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="K15" s="13" t="n">
         <v>705</v>
       </c>
-      <c r="L15" s="12">
+      <c r="L15" s="13">
         <f>I15*K15</f>
         <v/>
       </c>
-      <c r="M15" s="12">
+      <c r="M15" s="13">
         <f>L15*tc_actual</f>
         <v/>
       </c>
@@ -2080,30 +2103,30 @@
           <t>7.6 kW</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n">
+      <c r="F16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="10" t="n">
+      <c r="G16" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="H16" s="10" t="n">
+      <c r="H16" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="I16" s="10">
+      <c r="I16" s="11">
         <f>F16+G16-H16</f>
         <v/>
       </c>
-      <c r="J16" s="11" t="n">
+      <c r="J16" s="12" t="n">
         <v>0.1042</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="K16" s="13" t="n">
         <v>792</v>
       </c>
-      <c r="L16" s="12">
+      <c r="L16" s="13">
         <f>I16*K16</f>
         <v/>
       </c>
-      <c r="M16" s="12">
+      <c r="M16" s="13">
         <f>L16*tc_actual</f>
         <v/>
       </c>
@@ -2134,30 +2157,30 @@
           <t>9.6 kW</t>
         </is>
       </c>
-      <c r="F17" s="10" t="n">
+      <c r="F17" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="10" t="n">
+      <c r="G17" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="H17" s="10" t="n">
+      <c r="H17" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="I17" s="10">
+      <c r="I17" s="11">
         <f>F17+G17-H17</f>
         <v/>
       </c>
-      <c r="J17" s="11" t="n">
+      <c r="J17" s="12" t="n">
         <v>0.0936</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="K17" s="13" t="n">
         <v>899</v>
       </c>
-      <c r="L17" s="12">
+      <c r="L17" s="13">
         <f>I17*K17</f>
         <v/>
       </c>
-      <c r="M17" s="12">
+      <c r="M17" s="13">
         <f>L17*tc_actual</f>
         <v/>
       </c>
@@ -2188,28 +2211,28 @@
           <t>2 kW</t>
         </is>
       </c>
-      <c r="F18" s="10" t="n">
+      <c r="F18" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G18" s="10" t="n">
+      <c r="G18" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="10" t="n">
+      <c r="H18" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I18" s="10">
+      <c r="I18" s="11">
         <f>F18+G18-H18</f>
         <v/>
       </c>
-      <c r="J18" s="11" t="n"/>
-      <c r="K18" s="12" t="n">
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L18" s="12">
+      <c r="L18" s="13">
         <f>I18*K18</f>
         <v/>
       </c>
-      <c r="M18" s="12">
+      <c r="M18" s="13">
         <f>L18*tc_actual</f>
         <v/>
       </c>
@@ -2240,30 +2263,30 @@
           <t>15 kW</t>
         </is>
       </c>
-      <c r="F19" s="10" t="n">
+      <c r="F19" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="10" t="n">
+      <c r="G19" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="10" t="n">
+      <c r="H19" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I19" s="10">
+      <c r="I19" s="11">
         <f>F19+G19-H19</f>
         <v/>
       </c>
-      <c r="J19" s="11" t="n">
+      <c r="J19" s="12" t="n">
         <v>0.115</v>
       </c>
-      <c r="K19" s="12" t="n">
+      <c r="K19" s="13" t="n">
         <v>1725</v>
       </c>
-      <c r="L19" s="12">
+      <c r="L19" s="13">
         <f>I19*K19</f>
         <v/>
       </c>
-      <c r="M19" s="12">
+      <c r="M19" s="13">
         <f>L19*tc_actual</f>
         <v/>
       </c>
@@ -2294,30 +2317,30 @@
           <t>30 kW</t>
         </is>
       </c>
-      <c r="F20" s="10" t="n">
+      <c r="F20" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="10" t="n">
+      <c r="G20" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H20" s="10" t="n">
+      <c r="H20" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="I20" s="10">
+      <c r="I20" s="11">
         <f>F20+G20-H20</f>
         <v/>
       </c>
-      <c r="J20" s="11" t="n">
+      <c r="J20" s="12" t="n">
         <v>0.0779</v>
       </c>
-      <c r="K20" s="12" t="n">
+      <c r="K20" s="13" t="n">
         <v>2335.63</v>
       </c>
-      <c r="L20" s="12">
+      <c r="L20" s="13">
         <f>I20*K20</f>
         <v/>
       </c>
-      <c r="M20" s="12">
+      <c r="M20" s="13">
         <f>L20*tc_actual</f>
         <v/>
       </c>
@@ -2348,30 +2371,30 @@
           <t>36 kW</t>
         </is>
       </c>
-      <c r="F21" s="10" t="n">
+      <c r="F21" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="10" t="n">
+      <c r="G21" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H21" s="10" t="n">
+      <c r="H21" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="I21" s="10">
+      <c r="I21" s="11">
         <f>F21+G21-H21</f>
         <v/>
       </c>
-      <c r="J21" s="11" t="n">
+      <c r="J21" s="12" t="n">
         <v>0.0861</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="K21" s="13" t="n">
         <v>3098.45</v>
       </c>
-      <c r="L21" s="12">
+      <c r="L21" s="13">
         <f>I21*K21</f>
         <v/>
       </c>
-      <c r="M21" s="12">
+      <c r="M21" s="13">
         <f>L21*tc_actual</f>
         <v/>
       </c>
@@ -2402,28 +2425,28 @@
           <t>3 kW</t>
         </is>
       </c>
-      <c r="F22" s="10" t="n">
+      <c r="F22" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="10" t="n">
+      <c r="G22" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="10" t="n">
+      <c r="H22" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I22" s="10">
+      <c r="I22" s="11">
         <f>F22+G22-H22</f>
         <v/>
       </c>
-      <c r="J22" s="11" t="n"/>
-      <c r="K22" s="12" t="n">
+      <c r="J22" s="12" t="n"/>
+      <c r="K22" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L22" s="12">
+      <c r="L22" s="13">
         <f>I22*K22</f>
         <v/>
       </c>
-      <c r="M22" s="12">
+      <c r="M22" s="13">
         <f>L22*tc_actual</f>
         <v/>
       </c>
@@ -2454,30 +2477,30 @@
           <t>10 kW</t>
         </is>
       </c>
-      <c r="F23" s="10" t="n">
+      <c r="F23" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="10" t="n">
+      <c r="G23" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="H23" s="10" t="n">
+      <c r="H23" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="I23" s="10">
+      <c r="I23" s="11">
         <f>F23+G23-H23</f>
         <v/>
       </c>
-      <c r="J23" s="11" t="n">
+      <c r="J23" s="12" t="n">
         <v>0.094</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="K23" s="13" t="n">
         <v>940</v>
       </c>
-      <c r="L23" s="12">
+      <c r="L23" s="13">
         <f>I23*K23</f>
         <v/>
       </c>
-      <c r="M23" s="12">
+      <c r="M23" s="13">
         <f>L23*tc_actual</f>
         <v/>
       </c>
@@ -2508,30 +2531,30 @@
           <t>5 kW</t>
         </is>
       </c>
-      <c r="F24" s="10" t="n">
+      <c r="F24" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="G24" s="10" t="n">
+      <c r="G24" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="H24" s="10" t="n">
+      <c r="H24" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="I24" s="10">
+      <c r="I24" s="11">
         <f>F24+G24-H24</f>
         <v/>
       </c>
-      <c r="J24" s="11" t="n">
+      <c r="J24" s="12" t="n">
         <v>0.101</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="K24" s="13" t="n">
         <v>505</v>
       </c>
-      <c r="L24" s="12">
+      <c r="L24" s="13">
         <f>I24*K24</f>
         <v/>
       </c>
-      <c r="M24" s="12">
+      <c r="M24" s="13">
         <f>L24*tc_actual</f>
         <v/>
       </c>
@@ -2562,30 +2585,30 @@
           <t>6 kW</t>
         </is>
       </c>
-      <c r="F25" s="10" t="n">
+      <c r="F25" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="10" t="n">
+      <c r="G25" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="H25" s="10" t="n">
+      <c r="H25" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="I25" s="10">
+      <c r="I25" s="11">
         <f>F25+G25-H25</f>
         <v/>
       </c>
-      <c r="J25" s="11" t="n">
+      <c r="J25" s="12" t="n">
         <v>0.0883</v>
       </c>
-      <c r="K25" s="12" t="n">
+      <c r="K25" s="13" t="n">
         <v>530</v>
       </c>
-      <c r="L25" s="12">
+      <c r="L25" s="13">
         <f>I25*K25</f>
         <v/>
       </c>
-      <c r="M25" s="12">
+      <c r="M25" s="13">
         <f>L25*tc_actual</f>
         <v/>
       </c>
@@ -2616,30 +2639,30 @@
           <t>8 kW</t>
         </is>
       </c>
-      <c r="F26" s="10" t="n">
+      <c r="F26" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="10" t="n">
+      <c r="G26" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H26" s="10" t="n">
+      <c r="H26" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="I26" s="10">
+      <c r="I26" s="11">
         <f>F26+G26-H26</f>
         <v/>
       </c>
-      <c r="J26" s="11" t="n">
+      <c r="J26" s="12" t="n">
         <v>0.0919</v>
       </c>
-      <c r="K26" s="12" t="n">
+      <c r="K26" s="13" t="n">
         <v>735</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L26" s="13">
         <f>I26*K26</f>
         <v/>
       </c>
-      <c r="M26" s="12">
+      <c r="M26" s="13">
         <f>L26*tc_actual</f>
         <v/>
       </c>
@@ -2670,53 +2693,53 @@
           <t>3 kW</t>
         </is>
       </c>
-      <c r="F27" s="10" t="n">
+      <c r="F27" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="10" t="n">
+      <c r="G27" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="10" t="n">
+      <c r="H27" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I27" s="10">
+      <c r="I27" s="11">
         <f>F27+G27-H27</f>
         <v/>
       </c>
-      <c r="J27" s="11" t="n"/>
-      <c r="K27" s="12" t="n">
+      <c r="J27" s="12" t="n"/>
+      <c r="K27" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L27" s="12">
+      <c r="L27" s="13">
         <f>I27*K27</f>
         <v/>
       </c>
-      <c r="M27" s="12">
+      <c r="M27" s="13">
         <f>L27*tc_actual</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="n"/>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="A28" s="14" t="n"/>
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C28" s="13" t="n"/>
-      <c r="D28" s="13" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="13" t="n"/>
-      <c r="G28" s="13" t="n"/>
-      <c r="H28" s="13" t="n"/>
-      <c r="I28" s="13" t="n"/>
-      <c r="J28" s="13" t="n"/>
-      <c r="K28" s="13" t="n"/>
-      <c r="L28" s="14">
+      <c r="C28" s="14" t="n"/>
+      <c r="D28" s="14" t="n"/>
+      <c r="E28" s="14" t="n"/>
+      <c r="F28" s="14" t="n"/>
+      <c r="G28" s="14" t="n"/>
+      <c r="H28" s="14" t="n"/>
+      <c r="I28" s="14" t="n"/>
+      <c r="J28" s="14" t="n"/>
+      <c r="K28" s="14" t="n"/>
+      <c r="L28" s="15">
         <f>SUM(L2:L27)</f>
         <v/>
       </c>
-      <c r="M28" s="14">
+      <c r="M28" s="15">
         <f>SUM(M2:M27)</f>
         <v/>
       </c>
@@ -2815,27 +2838,27 @@
           <t>metros</t>
         </is>
       </c>
-      <c r="D2" s="10" t="n">
+      <c r="D2" s="11" t="n">
         <v>2600</v>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="E2" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="F2" s="11" t="n">
         <v>360</v>
       </c>
-      <c r="G2" s="10">
+      <c r="G2" s="11">
         <f>D2+E2-F2</f>
         <v/>
       </c>
-      <c r="H2" s="11" t="n">
+      <c r="H2" s="12" t="n">
         <v>0.8910761154855643</v>
       </c>
-      <c r="I2" s="12">
+      <c r="I2" s="13">
         <f>G2*H2</f>
         <v/>
       </c>
-      <c r="J2" s="12">
+      <c r="J2" s="13">
         <f>I2*tc_actual</f>
         <v/>
       </c>
@@ -2856,49 +2879,49 @@
           <t>metros</t>
         </is>
       </c>
-      <c r="D3" s="10" t="n">
+      <c r="D3" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="F3" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="11">
         <f>D3+E3-F3</f>
         <v/>
       </c>
-      <c r="H3" s="11" t="n">
+      <c r="H3" s="12" t="n">
         <v>0.8910761154855643</v>
       </c>
-      <c r="I3" s="12">
+      <c r="I3" s="13">
         <f>G3*H3</f>
         <v/>
       </c>
-      <c r="J3" s="12">
+      <c r="J3" s="13">
         <f>I3*tc_actual</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="n"/>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="n"/>
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C4" s="13" t="n"/>
-      <c r="D4" s="13" t="n"/>
-      <c r="E4" s="13" t="n"/>
-      <c r="F4" s="13" t="n"/>
-      <c r="G4" s="13" t="n"/>
-      <c r="H4" s="13" t="n"/>
-      <c r="I4" s="14">
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="14" t="n"/>
+      <c r="E4" s="14" t="n"/>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="14" t="n"/>
+      <c r="H4" s="14" t="n"/>
+      <c r="I4" s="15">
         <f>SUM(I2:I3)</f>
         <v/>
       </c>
-      <c r="J4" s="14">
+      <c r="J4" s="15">
         <f>SUM(J2:J3)</f>
         <v/>
       </c>
@@ -2914,17 +2937,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2945,25 +2970,35 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
+          <t>Cant. orig. (Excel)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>Precio unit. USD</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Color (origen)</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Etiqueta color</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Valor lote USD</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Valor lote MXN</t>
         </is>
@@ -2980,28 +3015,34 @@
           <t>1 Conector para riel inclinado</t>
         </is>
       </c>
-      <c r="C2" s="10" t="n">
+      <c r="C2" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="D2" s="11" t="n">
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr"/>
+      <c r="F2" s="12" t="n">
         <v>3.18</v>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F2" s="9" t="inlineStr">
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G2" s="12">
-        <f>C2*D2</f>
-        <v/>
-      </c>
-      <c r="H2" s="12">
-        <f>G2*tc_actual</f>
+      <c r="I2" s="13">
+        <f>C2*F2</f>
+        <v/>
+      </c>
+      <c r="J2" s="13">
+        <f>I2*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3016,28 +3057,34 @@
           <t>1 Conector para riel inclinado</t>
         </is>
       </c>
-      <c r="C3" s="10" t="n">
+      <c r="C3" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="D3" s="11" t="n">
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr"/>
+      <c r="F3" s="12" t="n">
         <v>3.18</v>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>theme:8</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>Color B</t>
         </is>
       </c>
-      <c r="G3" s="12">
-        <f>C3*D3</f>
-        <v/>
-      </c>
-      <c r="H3" s="12">
-        <f>G3*tc_actual</f>
+      <c r="I3" s="13">
+        <f>C3*F3</f>
+        <v/>
+      </c>
+      <c r="J3" s="13">
+        <f>I3*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3052,28 +3099,34 @@
           <t>1 Conector para riel inclinado</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="11" t="n">
         <v>315</v>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr"/>
+      <c r="F4" s="12" t="n">
         <v>3.16</v>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G4" s="12">
-        <f>C4*D4</f>
-        <v/>
-      </c>
-      <c r="H4" s="12">
-        <f>G4*tc_actual</f>
+      <c r="I4" s="13">
+        <f>C4*F4</f>
+        <v/>
+      </c>
+      <c r="J4" s="13">
+        <f>I4*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3088,28 +3141,34 @@
           <t>1 Conector para riel inclinado</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr"/>
+      <c r="F5" s="12" t="n">
         <v>3.18</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G5" s="12">
-        <f>C5*D5</f>
-        <v/>
-      </c>
-      <c r="H5" s="12">
-        <f>G5*tc_actual</f>
+      <c r="I5" s="13">
+        <f>C5*F5</f>
+        <v/>
+      </c>
+      <c r="J5" s="13">
+        <f>I5*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3124,28 +3183,34 @@
           <t>1 empalme de riel con puesta a tierra para Next Rail NXT-RX.</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr"/>
+      <c r="F6" s="12" t="n">
         <v>2.79</v>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G6" s="12">
-        <f>C6*D6</f>
-        <v/>
-      </c>
-      <c r="H6" s="12">
-        <f>G6*tc_actual</f>
+      <c r="I6" s="13">
+        <f>C6*F6</f>
+        <v/>
+      </c>
+      <c r="J6" s="13">
+        <f>I6*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3160,28 +3225,34 @@
           <t>1 empalme de riel con puesta a tierra para Next Rail NXT-RX.</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr"/>
+      <c r="F7" s="12" t="n">
         <v>2.79</v>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>theme:8</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>Color B</t>
         </is>
       </c>
-      <c r="G7" s="12">
-        <f>C7*D7</f>
-        <v/>
-      </c>
-      <c r="H7" s="12">
-        <f>G7*tc_actual</f>
+      <c r="I7" s="13">
+        <f>C7*F7</f>
+        <v/>
+      </c>
+      <c r="J7" s="13">
+        <f>I7*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3196,28 +3267,34 @@
           <t>1 empalme de riel con puesta a tierra para Next Rail NXT-RX.</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="11" t="n">
         <v>315</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="12" t="n">
         <v>2.78</v>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G8" s="12">
-        <f>C8*D8</f>
-        <v/>
-      </c>
-      <c r="H8" s="12">
-        <f>G8*tc_actual</f>
+      <c r="I8" s="13">
+        <f>C8*F8</f>
+        <v/>
+      </c>
+      <c r="J8" s="13">
+        <f>I8*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3232,28 +3309,34 @@
           <t>1 empalme de riel con puesta a tierra para Next Rail NXT-RX.</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr"/>
+      <c r="F9" s="12" t="n">
         <v>2.79</v>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G9" s="12">
-        <f>C9*D9</f>
-        <v/>
-      </c>
-      <c r="H9" s="12">
-        <f>G9*tc_actual</f>
+      <c r="I9" s="13">
+        <f>C9*F9</f>
+        <v/>
+      </c>
+      <c r="J9" s="13">
+        <f>I9*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3268,28 +3351,34 @@
           <t>1 Soporte "L" de 95 mm de altura para Nxt-Rail</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="11" t="n">
         <v>110</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr"/>
+      <c r="F10" s="12" t="n">
         <v>2.18</v>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G10" s="12">
-        <f>C10*D10</f>
-        <v/>
-      </c>
-      <c r="H10" s="12">
-        <f>G10*tc_actual</f>
+      <c r="I10" s="13">
+        <f>C10*F10</f>
+        <v/>
+      </c>
+      <c r="J10" s="13">
+        <f>I10*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3304,28 +3393,34 @@
           <t>1 Soporte "L" de 95 mm de altura para Nxt-Rail</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="11" t="n">
         <v>110</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr"/>
+      <c r="F11" s="12" t="n">
         <v>2.18</v>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>theme:8</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>Color B</t>
         </is>
       </c>
-      <c r="G11" s="12">
-        <f>C11*D11</f>
-        <v/>
-      </c>
-      <c r="H11" s="12">
-        <f>G11*tc_actual</f>
+      <c r="I11" s="13">
+        <f>C11*F11</f>
+        <v/>
+      </c>
+      <c r="J11" s="13">
+        <f>I11*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3340,28 +3435,34 @@
           <t>1 Soporte "L" de 95 mm de altura para Nxt-Rail</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="11" t="n">
         <v>315</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr"/>
+      <c r="F12" s="12" t="n">
         <v>2.17</v>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G12" s="12">
-        <f>C12*D12</f>
-        <v/>
-      </c>
-      <c r="H12" s="12">
-        <f>G12*tc_actual</f>
+      <c r="I12" s="13">
+        <f>C12*F12</f>
+        <v/>
+      </c>
+      <c r="J12" s="13">
+        <f>I12*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3376,28 +3477,34 @@
           <t>1 Soporte "L" de 95 mm de altura para Nxt-Rail</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="11" t="n">
         <v>110</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr"/>
+      <c r="F13" s="12" t="n">
         <v>2.18</v>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G13" s="12">
-        <f>C13*D13</f>
-        <v/>
-      </c>
-      <c r="H13" s="12">
-        <f>G13*tc_actual</f>
+      <c r="I13" s="13">
+        <f>C13*F13</f>
+        <v/>
+      </c>
+      <c r="J13" s="13">
+        <f>I13*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3412,28 +3519,34 @@
           <t>10 Conectores MC4, 5 Hembras y 5 Macho cable 14-10AWG, 1500 Vdc</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr"/>
+      <c r="F14" s="12" t="n">
         <v>5.56</v>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G14" s="12">
-        <f>C14*D14</f>
-        <v/>
-      </c>
-      <c r="H14" s="12">
-        <f>G14*tc_actual</f>
+      <c r="I14" s="13">
+        <f>C14*F14</f>
+        <v/>
+      </c>
+      <c r="J14" s="13">
+        <f>I14*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3448,28 +3561,34 @@
           <t>2 Abrazaderas universales de Aluminio para paneles de 30-46mm</t>
         </is>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="11" t="n">
         <v>910</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr"/>
+      <c r="F15" s="12" t="n">
         <v>3.99</v>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G15" s="12">
-        <f>C15*D15</f>
-        <v/>
-      </c>
-      <c r="H15" s="12">
-        <f>G15*tc_actual</f>
+      <c r="I15" s="13">
+        <f>C15*F15</f>
+        <v/>
+      </c>
+      <c r="J15" s="13">
+        <f>I15*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3484,28 +3603,34 @@
           <t>2 Abrazaderas universales de Aluminio para paneles de 30-46mm</t>
         </is>
       </c>
-      <c r="C16" s="10" t="n">
+      <c r="C16" s="11" t="n">
         <v>910</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr"/>
+      <c r="F16" s="12" t="n">
         <v>3.99</v>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>theme:8</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>Color B</t>
         </is>
       </c>
-      <c r="G16" s="12">
-        <f>C16*D16</f>
-        <v/>
-      </c>
-      <c r="H16" s="12">
-        <f>G16*tc_actual</f>
+      <c r="I16" s="13">
+        <f>C16*F16</f>
+        <v/>
+      </c>
+      <c r="J16" s="13">
+        <f>I16*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3520,28 +3645,34 @@
           <t>2 Abrazaderas universales de Aluminio para paneles de 30-46mm</t>
         </is>
       </c>
-      <c r="C17" s="10" t="n">
+      <c r="C17" s="11" t="n">
         <v>315</v>
       </c>
-      <c r="D17" s="11" t="n">
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr"/>
+      <c r="F17" s="12" t="n">
         <v>3.97</v>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G17" s="12">
-        <f>C17*D17</f>
-        <v/>
-      </c>
-      <c r="H17" s="12">
-        <f>G17*tc_actual</f>
+      <c r="I17" s="13">
+        <f>C17*F17</f>
+        <v/>
+      </c>
+      <c r="J17" s="13">
+        <f>I17*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3556,28 +3687,34 @@
           <t>2 Abrazaderas universales de Aluminio para paneles de 30-46mm</t>
         </is>
       </c>
-      <c r="C18" s="10" t="n">
+      <c r="C18" s="11" t="n">
         <v>910</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr"/>
+      <c r="F18" s="12" t="n">
         <v>3.99</v>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G18" s="12">
-        <f>C18*D18</f>
-        <v/>
-      </c>
-      <c r="H18" s="12">
-        <f>G18*tc_actual</f>
+      <c r="I18" s="13">
+        <f>C18*F18</f>
+        <v/>
+      </c>
+      <c r="J18" s="13">
+        <f>I18*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3592,28 +3729,34 @@
           <t>4 Clips de conexión para Next Rail</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr"/>
+      <c r="F19" s="12" t="n">
         <v>6.05</v>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G19" s="12">
-        <f>C19*D19</f>
-        <v/>
-      </c>
-      <c r="H19" s="12">
-        <f>G19*tc_actual</f>
+      <c r="I19" s="13">
+        <f>C19*F19</f>
+        <v/>
+      </c>
+      <c r="J19" s="13">
+        <f>I19*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3628,28 +3771,34 @@
           <t>4 Clips de conexión para Next Rail</t>
         </is>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="D20" s="11" t="n">
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr"/>
+      <c r="F20" s="12" t="n">
         <v>6.05</v>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="G20" s="9" t="inlineStr">
         <is>
           <t>theme:8</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="H20" s="9" t="inlineStr">
         <is>
           <t>Color B</t>
         </is>
       </c>
-      <c r="G20" s="12">
-        <f>C20*D20</f>
-        <v/>
-      </c>
-      <c r="H20" s="12">
-        <f>G20*tc_actual</f>
+      <c r="I20" s="13">
+        <f>C20*F20</f>
+        <v/>
+      </c>
+      <c r="J20" s="13">
+        <f>I20*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3664,28 +3813,34 @@
           <t>4 Clips de conexión para Next Rail</t>
         </is>
       </c>
-      <c r="C21" s="10" t="n">
+      <c r="C21" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="D21" s="11" t="n">
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr"/>
+      <c r="F21" s="12" t="n">
         <v>6.05</v>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G21" s="12">
-        <f>C21*D21</f>
-        <v/>
-      </c>
-      <c r="H21" s="12">
-        <f>G21*tc_actual</f>
+      <c r="I21" s="13">
+        <f>C21*F21</f>
+        <v/>
+      </c>
+      <c r="J21" s="13">
+        <f>I21*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3700,28 +3855,34 @@
           <t>5 Tbolt M8x25 Acero Inoxidable con tuerca para NextRail</t>
         </is>
       </c>
-      <c r="C22" s="10" t="n">
+      <c r="C22" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="D22" s="11" t="n">
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr"/>
+      <c r="F22" s="12" t="n">
         <v>2.47</v>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G22" s="12">
-        <f>C22*D22</f>
-        <v/>
-      </c>
-      <c r="H22" s="12">
-        <f>G22*tc_actual</f>
+      <c r="I22" s="13">
+        <f>C22*F22</f>
+        <v/>
+      </c>
+      <c r="J22" s="13">
+        <f>I22*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3736,28 +3897,34 @@
           <t>5 Tbolt M8x25 Acero Inoxidable con tuerca para NextRail</t>
         </is>
       </c>
-      <c r="C23" s="10" t="n">
+      <c r="C23" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="D23" s="11" t="n">
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr"/>
+      <c r="F23" s="12" t="n">
         <v>2.47</v>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>theme:8</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="H23" s="9" t="inlineStr">
         <is>
           <t>Color B</t>
         </is>
       </c>
-      <c r="G23" s="12">
-        <f>C23*D23</f>
-        <v/>
-      </c>
-      <c r="H23" s="12">
-        <f>G23*tc_actual</f>
+      <c r="I23" s="13">
+        <f>C23*F23</f>
+        <v/>
+      </c>
+      <c r="J23" s="13">
+        <f>I23*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3772,28 +3939,34 @@
           <t>5 Tbolt M8x25 Acero Inoxidable con tuerca para NextRail</t>
         </is>
       </c>
-      <c r="C24" s="10" t="n">
+      <c r="C24" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="D24" s="11" t="n">
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr"/>
+      <c r="F24" s="12" t="n">
         <v>2.47</v>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="H24" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G24" s="12">
-        <f>C24*D24</f>
-        <v/>
-      </c>
-      <c r="H24" s="12">
-        <f>G24*tc_actual</f>
+      <c r="I24" s="13">
+        <f>C24*F24</f>
+        <v/>
+      </c>
+      <c r="J24" s="13">
+        <f>I24*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3808,28 +3981,34 @@
           <t>Ángulo-Riel 4.0m, Alu 6105-T6</t>
         </is>
       </c>
-      <c r="C25" s="10" t="n">
+      <c r="C25" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="D25" s="11" t="n">
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr"/>
+      <c r="F25" s="12" t="n">
         <v>25.25</v>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="H25" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G25" s="12">
-        <f>C25*D25</f>
-        <v/>
-      </c>
-      <c r="H25" s="12">
-        <f>G25*tc_actual</f>
+      <c r="I25" s="13">
+        <f>C25*F25</f>
+        <v/>
+      </c>
+      <c r="J25" s="13">
+        <f>I25*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3844,28 +4023,34 @@
           <t>Ángulo-Riel 4.0m, Alu 6105-T6</t>
         </is>
       </c>
-      <c r="C26" s="10" t="n">
+      <c r="C26" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="D26" s="11" t="n">
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr"/>
+      <c r="F26" s="12" t="n">
         <v>25.25</v>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>theme:8</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr">
         <is>
           <t>Color B</t>
         </is>
       </c>
-      <c r="G26" s="12">
-        <f>C26*D26</f>
-        <v/>
-      </c>
-      <c r="H26" s="12">
-        <f>G26*tc_actual</f>
+      <c r="I26" s="13">
+        <f>C26*F26</f>
+        <v/>
+      </c>
+      <c r="J26" s="13">
+        <f>I26*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3880,28 +4065,34 @@
           <t>Ángulo-Riel 4.0m, Alu 6105-T6</t>
         </is>
       </c>
-      <c r="C27" s="10" t="n">
+      <c r="C27" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="D27" s="11" t="n">
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr"/>
+      <c r="F27" s="12" t="n">
         <v>25.25</v>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="H27" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G27" s="12">
-        <f>C27*D27</f>
-        <v/>
-      </c>
-      <c r="H27" s="12">
-        <f>G27*tc_actual</f>
+      <c r="I27" s="13">
+        <f>C27*F27</f>
+        <v/>
+      </c>
+      <c r="J27" s="13">
+        <f>I27*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3916,28 +4107,34 @@
           <t>Cable Fotovoltaico negro PV Wire carrete 762 mts 10AWG 2000V De 19 hilos</t>
         </is>
       </c>
-      <c r="C28" s="10" t="n">
+      <c r="C28" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="D28" s="11" t="n">
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr"/>
+      <c r="F28" s="12" t="n">
         <v>612.8200000000001</v>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="H28" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G28" s="12">
-        <f>C28*D28</f>
-        <v/>
-      </c>
-      <c r="H28" s="12">
-        <f>G28*tc_actual</f>
+      <c r="I28" s="13">
+        <f>C28*F28</f>
+        <v/>
+      </c>
+      <c r="J28" s="13">
+        <f>I28*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3952,28 +4149,34 @@
           <t>Cable Fotovoltaico negro PV Wire carrete 762 mts 10AWG 2000V De 19 hilos</t>
         </is>
       </c>
-      <c r="C29" s="10" t="n">
+      <c r="C29" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="D29" s="11" t="n">
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr"/>
+      <c r="F29" s="12" t="n">
         <v>612.8200000000001</v>
       </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="H29" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G29" s="12">
-        <f>C29*D29</f>
-        <v/>
-      </c>
-      <c r="H29" s="12">
-        <f>G29*tc_actual</f>
+      <c r="I29" s="13">
+        <f>C29*F29</f>
+        <v/>
+      </c>
+      <c r="J29" s="13">
+        <f>I29*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -3988,28 +4191,34 @@
           <t>Cable Fotovoltaico Negro PV wire carrete 762 mts 12AWG 2000V de 19 hilos</t>
         </is>
       </c>
-      <c r="C30" s="10" t="n">
+      <c r="C30" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="D30" s="11" t="n">
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr"/>
+      <c r="F30" s="12" t="n">
         <v>421.81</v>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="G30" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="H30" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G30" s="12">
-        <f>C30*D30</f>
-        <v/>
-      </c>
-      <c r="H30" s="12">
-        <f>G30*tc_actual</f>
+      <c r="I30" s="13">
+        <f>C30*F30</f>
+        <v/>
+      </c>
+      <c r="J30" s="13">
+        <f>I30*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -4024,28 +4233,34 @@
           <t>Cable Fotovoltaico Negro PV wire carrete 762 mts 12AWG 2000V de 19 hilos</t>
         </is>
       </c>
-      <c r="C31" s="10" t="n">
+      <c r="C31" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="D31" s="11" t="n">
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr"/>
+      <c r="F31" s="12" t="n">
         <v>421.81</v>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="G31" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="H31" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G31" s="12">
-        <f>C31*D31</f>
-        <v/>
-      </c>
-      <c r="H31" s="12">
-        <f>G31*tc_actual</f>
+      <c r="I31" s="13">
+        <f>C31*F31</f>
+        <v/>
+      </c>
+      <c r="J31" s="13">
+        <f>I31*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -4061,27 +4276,35 @@
         </is>
       </c>
       <c r="C32" s="10" t="n">
+        <v>1546</v>
+      </c>
+      <c r="D32" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="D32" s="11" t="n">
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>Cliente confirma 1546 paneles, no 15 (error de captura original)</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="n">
         <v>76.88</v>
       </c>
-      <c r="E32" s="9" t="inlineStr">
+      <c r="G32" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F32" s="9" t="inlineStr">
+      <c r="H32" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G32" s="12">
-        <f>C32*D32</f>
-        <v/>
-      </c>
-      <c r="H32" s="12">
-        <f>G32*tc_actual</f>
+      <c r="I32" s="13">
+        <f>C32*F32</f>
+        <v/>
+      </c>
+      <c r="J32" s="13">
+        <f>I32*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -4096,28 +4319,34 @@
           <t>Perfil NetRail 4.80m, mill finish, Aluminio 6105-T6</t>
         </is>
       </c>
-      <c r="C33" s="10" t="n">
+      <c r="C33" s="11" t="n">
         <v>245</v>
       </c>
-      <c r="D33" s="11" t="n">
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr"/>
+      <c r="F33" s="12" t="n">
         <v>25.64</v>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="G33" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="H33" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G33" s="12">
-        <f>C33*D33</f>
-        <v/>
-      </c>
-      <c r="H33" s="12">
-        <f>G33*tc_actual</f>
+      <c r="I33" s="13">
+        <f>C33*F33</f>
+        <v/>
+      </c>
+      <c r="J33" s="13">
+        <f>I33*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -4132,28 +4361,34 @@
           <t>Perfil NetRail 4.80m, mill finish, Aluminio 6105-T6</t>
         </is>
       </c>
-      <c r="C34" s="10" t="n">
+      <c r="C34" s="11" t="n">
         <v>245</v>
       </c>
-      <c r="D34" s="11" t="n">
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr"/>
+      <c r="F34" s="12" t="n">
         <v>25.64</v>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="G34" s="9" t="inlineStr">
         <is>
           <t>theme:8</t>
         </is>
       </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="H34" s="9" t="inlineStr">
         <is>
           <t>Color B</t>
         </is>
       </c>
-      <c r="G34" s="12">
-        <f>C34*D34</f>
-        <v/>
-      </c>
-      <c r="H34" s="12">
-        <f>G34*tc_actual</f>
+      <c r="I34" s="13">
+        <f>C34*F34</f>
+        <v/>
+      </c>
+      <c r="J34" s="13">
+        <f>I34*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -4168,28 +4403,34 @@
           <t>Perfil NetRail 4.80m, mill finish, Aluminio 6105-T6</t>
         </is>
       </c>
-      <c r="C35" s="10" t="n">
+      <c r="C35" s="11" t="n">
         <v>385</v>
       </c>
-      <c r="D35" s="11" t="n">
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr"/>
+      <c r="F35" s="12" t="n">
         <v>25.51</v>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="G35" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="H35" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G35" s="12">
-        <f>C35*D35</f>
-        <v/>
-      </c>
-      <c r="H35" s="12">
-        <f>G35*tc_actual</f>
+      <c r="I35" s="13">
+        <f>C35*F35</f>
+        <v/>
+      </c>
+      <c r="J35" s="13">
+        <f>I35*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -4204,28 +4445,34 @@
           <t>Perfil NetRail 4.80m, mill finish, Aluminio 6105-T6</t>
         </is>
       </c>
-      <c r="C36" s="10" t="n">
+      <c r="C36" s="11" t="n">
         <v>245</v>
       </c>
-      <c r="D36" s="11" t="n">
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr"/>
+      <c r="F36" s="12" t="n">
         <v>25.64</v>
       </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="G36" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F36" s="9" t="inlineStr">
+      <c r="H36" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G36" s="12">
-        <f>C36*D36</f>
-        <v/>
-      </c>
-      <c r="H36" s="12">
-        <f>G36*tc_actual</f>
+      <c r="I36" s="13">
+        <f>C36*F36</f>
+        <v/>
+      </c>
+      <c r="J36" s="13">
+        <f>I36*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -4240,28 +4487,34 @@
           <t>Terminal de conexión a tierra para 2 cables, Next Rail con certificiación UL.</t>
         </is>
       </c>
-      <c r="C37" s="10" t="n">
+      <c r="C37" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="D37" s="11" t="n">
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr"/>
+      <c r="F37" s="12" t="n">
         <v>2.19</v>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="G37" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="H37" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G37" s="12">
-        <f>C37*D37</f>
-        <v/>
-      </c>
-      <c r="H37" s="12">
-        <f>G37*tc_actual</f>
+      <c r="I37" s="13">
+        <f>C37*F37</f>
+        <v/>
+      </c>
+      <c r="J37" s="13">
+        <f>I37*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -4276,28 +4529,34 @@
           <t>Terminal de conexión a tierra para 2 cables, Next Rail con certificiación UL.</t>
         </is>
       </c>
-      <c r="C38" s="10" t="n">
+      <c r="C38" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="D38" s="11" t="n">
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr"/>
+      <c r="F38" s="12" t="n">
         <v>2.19</v>
       </c>
-      <c r="E38" s="9" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr">
         <is>
           <t>theme:8</t>
         </is>
       </c>
-      <c r="F38" s="9" t="inlineStr">
+      <c r="H38" s="9" t="inlineStr">
         <is>
           <t>Color B</t>
         </is>
       </c>
-      <c r="G38" s="12">
-        <f>C38*D38</f>
-        <v/>
-      </c>
-      <c r="H38" s="12">
-        <f>G38*tc_actual</f>
+      <c r="I38" s="13">
+        <f>C38*F38</f>
+        <v/>
+      </c>
+      <c r="J38" s="13">
+        <f>I38*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -4312,28 +4571,34 @@
           <t>Terminal de conexión a tierra para 2 cables, Next Rail con certificiación UL.</t>
         </is>
       </c>
-      <c r="C39" s="10" t="n">
+      <c r="C39" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="D39" s="11" t="n">
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr"/>
+      <c r="F39" s="12" t="n">
         <v>2.19</v>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="G39" s="9" t="inlineStr">
         <is>
           <t>theme:9</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
+      <c r="H39" s="9" t="inlineStr">
         <is>
           <t>Color A (lote más frecuente)</t>
         </is>
       </c>
-      <c r="G39" s="12">
-        <f>C39*D39</f>
-        <v/>
-      </c>
-      <c r="H39" s="12">
-        <f>G39*tc_actual</f>
+      <c r="I39" s="13">
+        <f>C39*F39</f>
+        <v/>
+      </c>
+      <c r="J39" s="13">
+        <f>I39*tc_actual</f>
         <v/>
       </c>
     </row>
@@ -4348,48 +4613,56 @@
           <t>Terminal de conexión a tierra para 2 cables, Next Rail con certificiación UL.</t>
         </is>
       </c>
-      <c r="C40" s="10" t="n">
+      <c r="C40" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="D40" s="11" t="n">
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr"/>
+      <c r="F40" s="12" t="n">
         <v>2.19</v>
       </c>
-      <c r="E40" s="9" t="inlineStr">
+      <c r="G40" s="9" t="inlineStr">
         <is>
           <t>FFFFFF00</t>
         </is>
       </c>
-      <c r="F40" s="9" t="inlineStr">
+      <c r="H40" s="9" t="inlineStr">
         <is>
           <t>Color C (amarillo)</t>
         </is>
       </c>
-      <c r="G40" s="12">
-        <f>C40*D40</f>
-        <v/>
-      </c>
-      <c r="H40" s="12">
-        <f>G40*tc_actual</f>
+      <c r="I40" s="13">
+        <f>C40*F40</f>
+        <v/>
+      </c>
+      <c r="J40" s="13">
+        <f>I40*tc_actual</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="n"/>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="A41" s="14" t="n"/>
+      <c r="B41" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C41" s="13" t="n"/>
-      <c r="D41" s="13" t="n"/>
-      <c r="E41" s="13" t="n"/>
-      <c r="F41" s="13" t="n"/>
-      <c r="G41" s="14">
-        <f>SUM(G2:G40)</f>
-        <v/>
-      </c>
-      <c r="H41" s="14">
-        <f>SUM(H2:H40)</f>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="14" t="n"/>
+      <c r="E41" s="14" t="n"/>
+      <c r="F41" s="14" t="n"/>
+      <c r="G41" s="14" t="n"/>
+      <c r="H41" s="14" t="n"/>
+      <c r="I41" s="15">
+        <f>SUM(I2:I40)</f>
+        <v/>
+      </c>
+      <c r="J41" s="15">
+        <f>SUM(J2:J40)</f>
         <v/>
       </c>
     </row>

</xml_diff>